<commit_message>
WIP: Syncing to main
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/STAFFS-BUDDY-UP-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/STAFFS-BUDDY-UP-TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OSH TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A550E602-BA78-4526-A0BB-5E7C6F05EBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A808DB-74C4-4AFF-B691-6FC872086301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Staff Code</t>
   </si>
@@ -33,22 +33,19 @@
     <t>Effectivity Date</t>
   </si>
   <si>
-    <t>*Date should be formatted as d/m/y</t>
-  </si>
-  <si>
-    <t>* delete this line and above sample data on actual uploading</t>
-  </si>
-  <si>
-    <t>Store</t>
-  </si>
-  <si>
     <t>End Date</t>
   </si>
   <si>
+    <t>V211013-000005</t>
+  </si>
+  <si>
     <t>V211028-000004</t>
   </si>
   <si>
-    <t>GINGOOG 2</t>
+    <t>ZONE 5 BULUA CDO</t>
+  </si>
+  <si>
+    <t>New Store</t>
   </si>
 </sst>
 </file>
@@ -453,21 +450,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2">
         <v>46230</v>
@@ -476,15 +473,22 @@
         <v>46233</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
+    <row r="3" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46230</v>
+      </c>
+      <c r="D3" s="2">
+        <v>46233</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="A4" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Validation and Import Staff Transaction
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/STAFFS-BUDDY-UP-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/STAFFS-BUDDY-UP-TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OSH TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A808DB-74C4-4AFF-B691-6FC872086301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8434C07B-13D7-4D56-9ECE-F859C81CF926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Staff Code</t>
   </si>
@@ -33,16 +33,19 @@
     <t>Effectivity Date</t>
   </si>
   <si>
+    <t>*Date should be formatted as d/m/y</t>
+  </si>
+  <si>
+    <t>* delete this line and above sample data on actual uploading</t>
+  </si>
+  <si>
     <t>End Date</t>
   </si>
   <si>
-    <t>V211013-000005</t>
-  </si>
-  <si>
-    <t>V211028-000004</t>
-  </si>
-  <si>
-    <t>ZONE 5 BULUA CDO</t>
+    <t>NAGA - CENTRO</t>
+  </si>
+  <si>
+    <t>V211013-000004</t>
   </si>
   <si>
     <t>New Store</t>
@@ -118,10 +121,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,7 +441,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
     <col min="3" max="3" width="38.5703125" customWidth="1"/>
     <col min="4" max="4" width="37.28515625" customWidth="1"/>
   </cols>
@@ -450,18 +451,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
+      <c r="A2" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -473,22 +474,15 @@
         <v>46233</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2">
-        <v>46230</v>
-      </c>
-      <c r="D3" s="2">
-        <v>46233</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>